<commit_message>
Various Bugs Fixed/New design in gifts added
1. Import customer list bug still there
</commit_message>
<xml_diff>
--- a/bin/Release/Assets/Templates/temp_data.xlsx
+++ b/bin/Release/Assets/Templates/temp_data.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Συμμετέχων</t>
   </si>
@@ -36,6 +36,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>2310403354</t>
   </si>
   <si>
     <t>POWERTECH EARPHONES ME ΘΗΚΗ ΦΟΡΤΙΣΗΣ ΜΑΥΡΟ</t>
@@ -116,11 +119,11 @@
         <v>7</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2"/>
       <c r="F2" s="0" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>